<commit_message>
Commit with untracked changes and changes with Excel
</commit_message>
<xml_diff>
--- a/Resources/TestcasesCartOffer.xlsx
+++ b/Resources/TestcasesCartOffer.xlsx
@@ -8,14 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Code\ZomatoCartOfferAPI\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84A86A2F-C097-4AA0-A82E-458A61BAB45B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31305188-1BD3-4927-A12C-8742EC143116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TestData_CartOffer" sheetId="2" r:id="rId1"/>
     <sheet name="API Mappings" sheetId="3" r:id="rId2"/>
-    <sheet name="BDD validations" sheetId="1" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,41 +26,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="35">
-  <si>
-    <t>TC ID</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="27">
   <si>
     <t>Scenario</t>
   </si>
   <si>
-    <t>Pre-requisite</t>
-  </si>
-  <si>
-    <t>Given</t>
-  </si>
-  <si>
-    <t>When</t>
-  </si>
-  <si>
-    <t>Then</t>
-  </si>
-  <si>
-    <t>Pass/Fail</t>
-  </si>
-  <si>
-    <t>Verify that the API response status code is 200 OK</t>
-  </si>
-  <si>
-    <t>Verify that the API response is in the expected format (e.g. JSON, XML).</t>
-  </si>
-  <si>
-    <t>Verify that the API response contains all the expected fields.</t>
-  </si>
-  <si>
-    <t>Verify that the API response contains the correct data for each field</t>
-  </si>
-  <si>
     <t>OfferType</t>
   </si>
   <si>
@@ -119,9 +88,6 @@
     <t>Negetive scenario: Invalid segment</t>
   </si>
   <si>
-    <t>Positive scenario</t>
-  </si>
-  <si>
     <t>Restaurant_id</t>
   </si>
   <si>
@@ -132,6 +98,15 @@
   </si>
   <si>
     <t>UserId and segmentId mapping</t>
+  </si>
+  <si>
+    <t>Positive scenario for P1 segment</t>
+  </si>
+  <si>
+    <t>Positive scenario for P2 segment</t>
+  </si>
+  <si>
+    <t>Positive scenario for P3 segment</t>
   </si>
 </sst>
 </file>
@@ -184,10 +159,10 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -479,16 +454,19 @@
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>16</v>
+        <v>6</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -505,7 +483,7 @@
         <v>190</v>
       </c>
       <c r="E2" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -522,7 +500,7 @@
         <v>95</v>
       </c>
       <c r="E3" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -539,7 +517,7 @@
         <v>400</v>
       </c>
       <c r="E4" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -556,7 +534,7 @@
         <v>125</v>
       </c>
       <c r="E5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -573,7 +551,7 @@
         <v>200</v>
       </c>
       <c r="E6" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -590,7 +568,7 @@
         <v>1000</v>
       </c>
       <c r="E7" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -607,14 +585,14 @@
         <v>200</v>
       </c>
       <c r="E8" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H14" s="3"/>
+      <c r="H14" s="2"/>
     </row>
     <row r="15" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H15" s="3"/>
+      <c r="H15" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -632,26 +610,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
+      <c r="A1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -659,13 +637,13 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C3">
         <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -673,13 +651,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C4">
         <v>5</v>
       </c>
       <c r="D4" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -687,13 +665,13 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C5">
         <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -701,13 +679,13 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C6">
         <v>25</v>
       </c>
       <c r="D6" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -715,13 +693,13 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C7">
         <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -729,13 +707,13 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C8">
         <v>30</v>
       </c>
       <c r="D8" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -743,27 +721,27 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C9">
         <v>30</v>
       </c>
       <c r="D9" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="2"/>
+      <c r="A13" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="3"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -771,7 +749,7 @@
         <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -779,7 +757,7 @@
         <v>2</v>
       </c>
       <c r="B16" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -787,7 +765,7 @@
         <v>3</v>
       </c>
       <c r="B17" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -795,7 +773,7 @@
         <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -803,7 +781,7 @@
         <v>5</v>
       </c>
       <c r="B19" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -811,7 +789,7 @@
         <v>6</v>
       </c>
       <c r="B20" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -819,7 +797,7 @@
         <v>2</v>
       </c>
       <c r="B21" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -829,62 +807,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="65.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
-        <v>10</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>